<commit_message>
Add FOB to Cost Type dropdown options
Cost Type now: Landed, DDP, DAP, FOB

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/PRD_Research_Template.xlsx
+++ b/templates/PRD_Research_Template.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ideations" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ideations'!$A$2:$AZ$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ideations'!$A$2:$BA$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -686,21 +686,21 @@
     <row r="29">
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>BUSINESS TARGETS (Columns AQ–AW)</t>
+          <t>BUSINESS TARGETS (Columns AQ–AX)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Pricing targets (MSRP, margin, vendor cost), certifications,</t>
+          <t xml:space="preserve">  Pricing targets (MSRP, margin), cost type (Landed/DDP/DAP),</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  rated lifetime, and warranty period.</t>
+          <t xml:space="preserve">  vendor cost, certifications, rated lifetime, and warranty.</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
     <row r="33">
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>RESEARCH GUIDANCE (Columns AX–AZ)</t>
+          <t>RESEARCH GUIDANCE (Columns AY–BA)</t>
         </is>
       </c>
     </row>
@@ -782,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ102"/>
+  <dimension ref="A1:BA102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -834,9 +834,10 @@
     <col width="16" customWidth="1" min="47" max="47"/>
     <col width="16" customWidth="1" min="48" max="48"/>
     <col width="16" customWidth="1" min="49" max="49"/>
-    <col width="22" customWidth="1" min="50" max="50"/>
+    <col width="16" customWidth="1" min="50" max="50"/>
     <col width="22" customWidth="1" min="51" max="51"/>
     <col width="22" customWidth="1" min="52" max="52"/>
+    <col width="22" customWidth="1" min="53" max="53"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -909,13 +910,14 @@
       <c r="AU1" s="1" t="n"/>
       <c r="AV1" s="1" t="n"/>
       <c r="AW1" s="1" t="n"/>
-      <c r="AX1" s="6" t="inlineStr">
+      <c r="AX1" s="1" t="n"/>
+      <c r="AY1" s="6" t="inlineStr">
         <is>
           <t>RESEARCH GUIDANCE</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="n"/>
       <c r="AZ1" s="1" t="n"/>
+      <c r="BA1" s="1" t="n"/>
     </row>
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
@@ -1145,35 +1147,40 @@
       </c>
       <c r="AT2" s="8" t="inlineStr">
         <is>
+          <t>Cost Type</t>
+        </is>
+      </c>
+      <c r="AU2" s="8" t="inlineStr">
+        <is>
           <t>Target Vendor Cost</t>
         </is>
       </c>
-      <c r="AU2" s="8" t="inlineStr">
+      <c r="AV2" s="8" t="inlineStr">
         <is>
           <t>Certifications</t>
         </is>
       </c>
-      <c r="AV2" s="8" t="inlineStr">
+      <c r="AW2" s="8" t="inlineStr">
         <is>
           <t>Lifetime Hours</t>
         </is>
       </c>
-      <c r="AW2" s="8" t="inlineStr">
+      <c r="AX2" s="8" t="inlineStr">
         <is>
           <t>Warranty</t>
         </is>
       </c>
-      <c r="AX2" s="8" t="inlineStr">
+      <c r="AY2" s="8" t="inlineStr">
         <is>
           <t>Known Competitors</t>
         </is>
       </c>
-      <c r="AY2" s="8" t="inlineStr">
+      <c r="AZ2" s="8" t="inlineStr">
         <is>
           <t>Priority Channels</t>
         </is>
       </c>
-      <c r="AZ2" s="8" t="inlineStr">
+      <c r="BA2" s="8" t="inlineStr">
         <is>
           <t>Research Notes</t>
         </is>
@@ -1387,35 +1394,40 @@
       </c>
       <c r="AT3" s="9" t="inlineStr">
         <is>
+          <t>Landed</t>
+        </is>
+      </c>
+      <c r="AU3" s="9" t="inlineStr">
+        <is>
           <t>$18.00</t>
         </is>
       </c>
-      <c r="AU3" s="9" t="inlineStr">
+      <c r="AV3" s="9" t="inlineStr">
         <is>
           <t>UL, DLC, FCC, Energy Star</t>
         </is>
       </c>
-      <c r="AV3" s="9" t="inlineStr">
+      <c r="AW3" s="9" t="inlineStr">
         <is>
           <t>50,000</t>
         </is>
       </c>
-      <c r="AW3" s="9" t="inlineStr">
+      <c r="AX3" s="9" t="inlineStr">
         <is>
           <t>7-Year</t>
         </is>
       </c>
-      <c r="AX3" s="9" t="inlineStr">
+      <c r="AY3" s="9" t="inlineStr">
         <is>
           <t>Metalux, Lithonia, TCP</t>
         </is>
       </c>
-      <c r="AY3" s="9" t="inlineStr">
+      <c r="AZ3" s="9" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="AZ3" s="9" t="inlineStr">
+      <c r="BA3" s="9" t="inlineStr">
         <is>
           <t>High-output selectable wattage panel to replace PN24-2x4-30W line. Target DLC Premium for utility rebates.</t>
         </is>
@@ -1474,6 +1486,7 @@
       <c r="AX4" s="10" t="n"/>
       <c r="AY4" s="10" t="n"/>
       <c r="AZ4" s="10" t="n"/>
+      <c r="BA4" s="10" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n"/>
@@ -1528,6 +1541,7 @@
       <c r="AX5" s="9" t="n"/>
       <c r="AY5" s="9" t="n"/>
       <c r="AZ5" s="9" t="n"/>
+      <c r="BA5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="10" t="n"/>
@@ -1582,6 +1596,7 @@
       <c r="AX6" s="10" t="n"/>
       <c r="AY6" s="10" t="n"/>
       <c r="AZ6" s="10" t="n"/>
+      <c r="BA6" s="10" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n"/>
@@ -1636,6 +1651,7 @@
       <c r="AX7" s="9" t="n"/>
       <c r="AY7" s="9" t="n"/>
       <c r="AZ7" s="9" t="n"/>
+      <c r="BA7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="n"/>
@@ -1690,6 +1706,7 @@
       <c r="AX8" s="10" t="n"/>
       <c r="AY8" s="10" t="n"/>
       <c r="AZ8" s="10" t="n"/>
+      <c r="BA8" s="10" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="n"/>
@@ -1744,6 +1761,7 @@
       <c r="AX9" s="9" t="n"/>
       <c r="AY9" s="9" t="n"/>
       <c r="AZ9" s="9" t="n"/>
+      <c r="BA9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="n"/>
@@ -1798,6 +1816,7 @@
       <c r="AX10" s="10" t="n"/>
       <c r="AY10" s="10" t="n"/>
       <c r="AZ10" s="10" t="n"/>
+      <c r="BA10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n"/>
@@ -1852,6 +1871,7 @@
       <c r="AX11" s="9" t="n"/>
       <c r="AY11" s="9" t="n"/>
       <c r="AZ11" s="9" t="n"/>
+      <c r="BA11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="n"/>
@@ -1906,6 +1926,7 @@
       <c r="AX12" s="10" t="n"/>
       <c r="AY12" s="10" t="n"/>
       <c r="AZ12" s="10" t="n"/>
+      <c r="BA12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n"/>
@@ -1960,6 +1981,7 @@
       <c r="AX13" s="9" t="n"/>
       <c r="AY13" s="9" t="n"/>
       <c r="AZ13" s="9" t="n"/>
+      <c r="BA13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="n"/>
@@ -2014,6 +2036,7 @@
       <c r="AX14" s="10" t="n"/>
       <c r="AY14" s="10" t="n"/>
       <c r="AZ14" s="10" t="n"/>
+      <c r="BA14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n"/>
@@ -2068,6 +2091,7 @@
       <c r="AX15" s="9" t="n"/>
       <c r="AY15" s="9" t="n"/>
       <c r="AZ15" s="9" t="n"/>
+      <c r="BA15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n"/>
@@ -2122,6 +2146,7 @@
       <c r="AX16" s="10" t="n"/>
       <c r="AY16" s="10" t="n"/>
       <c r="AZ16" s="10" t="n"/>
+      <c r="BA16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="n"/>
@@ -2176,6 +2201,7 @@
       <c r="AX17" s="9" t="n"/>
       <c r="AY17" s="9" t="n"/>
       <c r="AZ17" s="9" t="n"/>
+      <c r="BA17" s="9" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n"/>
@@ -2230,6 +2256,7 @@
       <c r="AX18" s="10" t="n"/>
       <c r="AY18" s="10" t="n"/>
       <c r="AZ18" s="10" t="n"/>
+      <c r="BA18" s="10" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="n"/>
@@ -2284,6 +2311,7 @@
       <c r="AX19" s="9" t="n"/>
       <c r="AY19" s="9" t="n"/>
       <c r="AZ19" s="9" t="n"/>
+      <c r="BA19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n"/>
@@ -2338,6 +2366,7 @@
       <c r="AX20" s="10" t="n"/>
       <c r="AY20" s="10" t="n"/>
       <c r="AZ20" s="10" t="n"/>
+      <c r="BA20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="9" t="n"/>
@@ -2392,6 +2421,7 @@
       <c r="AX21" s="9" t="n"/>
       <c r="AY21" s="9" t="n"/>
       <c r="AZ21" s="9" t="n"/>
+      <c r="BA21" s="9" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n"/>
@@ -2446,6 +2476,7 @@
       <c r="AX22" s="10" t="n"/>
       <c r="AY22" s="10" t="n"/>
       <c r="AZ22" s="10" t="n"/>
+      <c r="BA22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="9" t="n"/>
@@ -2500,6 +2531,7 @@
       <c r="AX23" s="9" t="n"/>
       <c r="AY23" s="9" t="n"/>
       <c r="AZ23" s="9" t="n"/>
+      <c r="BA23" s="9" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n"/>
@@ -2554,6 +2586,7 @@
       <c r="AX24" s="10" t="n"/>
       <c r="AY24" s="10" t="n"/>
       <c r="AZ24" s="10" t="n"/>
+      <c r="BA24" s="10" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="9" t="n"/>
@@ -2608,6 +2641,7 @@
       <c r="AX25" s="9" t="n"/>
       <c r="AY25" s="9" t="n"/>
       <c r="AZ25" s="9" t="n"/>
+      <c r="BA25" s="9" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n"/>
@@ -2662,6 +2696,7 @@
       <c r="AX26" s="10" t="n"/>
       <c r="AY26" s="10" t="n"/>
       <c r="AZ26" s="10" t="n"/>
+      <c r="BA26" s="10" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="9" t="n"/>
@@ -2716,6 +2751,7 @@
       <c r="AX27" s="9" t="n"/>
       <c r="AY27" s="9" t="n"/>
       <c r="AZ27" s="9" t="n"/>
+      <c r="BA27" s="9" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n"/>
@@ -2770,6 +2806,7 @@
       <c r="AX28" s="10" t="n"/>
       <c r="AY28" s="10" t="n"/>
       <c r="AZ28" s="10" t="n"/>
+      <c r="BA28" s="10" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n"/>
@@ -2824,6 +2861,7 @@
       <c r="AX29" s="9" t="n"/>
       <c r="AY29" s="9" t="n"/>
       <c r="AZ29" s="9" t="n"/>
+      <c r="BA29" s="9" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n"/>
@@ -2878,6 +2916,7 @@
       <c r="AX30" s="10" t="n"/>
       <c r="AY30" s="10" t="n"/>
       <c r="AZ30" s="10" t="n"/>
+      <c r="BA30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="9" t="n"/>
@@ -2932,6 +2971,7 @@
       <c r="AX31" s="9" t="n"/>
       <c r="AY31" s="9" t="n"/>
       <c r="AZ31" s="9" t="n"/>
+      <c r="BA31" s="9" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n"/>
@@ -2986,6 +3026,7 @@
       <c r="AX32" s="10" t="n"/>
       <c r="AY32" s="10" t="n"/>
       <c r="AZ32" s="10" t="n"/>
+      <c r="BA32" s="10" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="9" t="n"/>
@@ -3040,6 +3081,7 @@
       <c r="AX33" s="9" t="n"/>
       <c r="AY33" s="9" t="n"/>
       <c r="AZ33" s="9" t="n"/>
+      <c r="BA33" s="9" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="n"/>
@@ -3094,6 +3136,7 @@
       <c r="AX34" s="10" t="n"/>
       <c r="AY34" s="10" t="n"/>
       <c r="AZ34" s="10" t="n"/>
+      <c r="BA34" s="10" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="9" t="n"/>
@@ -3148,6 +3191,7 @@
       <c r="AX35" s="9" t="n"/>
       <c r="AY35" s="9" t="n"/>
       <c r="AZ35" s="9" t="n"/>
+      <c r="BA35" s="9" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="n"/>
@@ -3202,6 +3246,7 @@
       <c r="AX36" s="10" t="n"/>
       <c r="AY36" s="10" t="n"/>
       <c r="AZ36" s="10" t="n"/>
+      <c r="BA36" s="10" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="9" t="n"/>
@@ -3256,6 +3301,7 @@
       <c r="AX37" s="9" t="n"/>
       <c r="AY37" s="9" t="n"/>
       <c r="AZ37" s="9" t="n"/>
+      <c r="BA37" s="9" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="n"/>
@@ -3310,6 +3356,7 @@
       <c r="AX38" s="10" t="n"/>
       <c r="AY38" s="10" t="n"/>
       <c r="AZ38" s="10" t="n"/>
+      <c r="BA38" s="10" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="9" t="n"/>
@@ -3364,6 +3411,7 @@
       <c r="AX39" s="9" t="n"/>
       <c r="AY39" s="9" t="n"/>
       <c r="AZ39" s="9" t="n"/>
+      <c r="BA39" s="9" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="n"/>
@@ -3418,6 +3466,7 @@
       <c r="AX40" s="10" t="n"/>
       <c r="AY40" s="10" t="n"/>
       <c r="AZ40" s="10" t="n"/>
+      <c r="BA40" s="10" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="9" t="n"/>
@@ -3472,6 +3521,7 @@
       <c r="AX41" s="9" t="n"/>
       <c r="AY41" s="9" t="n"/>
       <c r="AZ41" s="9" t="n"/>
+      <c r="BA41" s="9" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="10" t="n"/>
@@ -3526,6 +3576,7 @@
       <c r="AX42" s="10" t="n"/>
       <c r="AY42" s="10" t="n"/>
       <c r="AZ42" s="10" t="n"/>
+      <c r="BA42" s="10" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="9" t="n"/>
@@ -3580,6 +3631,7 @@
       <c r="AX43" s="9" t="n"/>
       <c r="AY43" s="9" t="n"/>
       <c r="AZ43" s="9" t="n"/>
+      <c r="BA43" s="9" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="10" t="n"/>
@@ -3634,6 +3686,7 @@
       <c r="AX44" s="10" t="n"/>
       <c r="AY44" s="10" t="n"/>
       <c r="AZ44" s="10" t="n"/>
+      <c r="BA44" s="10" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="9" t="n"/>
@@ -3688,6 +3741,7 @@
       <c r="AX45" s="9" t="n"/>
       <c r="AY45" s="9" t="n"/>
       <c r="AZ45" s="9" t="n"/>
+      <c r="BA45" s="9" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="10" t="n"/>
@@ -3742,6 +3796,7 @@
       <c r="AX46" s="10" t="n"/>
       <c r="AY46" s="10" t="n"/>
       <c r="AZ46" s="10" t="n"/>
+      <c r="BA46" s="10" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="9" t="n"/>
@@ -3796,6 +3851,7 @@
       <c r="AX47" s="9" t="n"/>
       <c r="AY47" s="9" t="n"/>
       <c r="AZ47" s="9" t="n"/>
+      <c r="BA47" s="9" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="10" t="n"/>
@@ -3850,6 +3906,7 @@
       <c r="AX48" s="10" t="n"/>
       <c r="AY48" s="10" t="n"/>
       <c r="AZ48" s="10" t="n"/>
+      <c r="BA48" s="10" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="9" t="n"/>
@@ -3904,6 +3961,7 @@
       <c r="AX49" s="9" t="n"/>
       <c r="AY49" s="9" t="n"/>
       <c r="AZ49" s="9" t="n"/>
+      <c r="BA49" s="9" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="10" t="n"/>
@@ -3958,6 +4016,7 @@
       <c r="AX50" s="10" t="n"/>
       <c r="AY50" s="10" t="n"/>
       <c r="AZ50" s="10" t="n"/>
+      <c r="BA50" s="10" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="9" t="n"/>
@@ -4012,6 +4071,7 @@
       <c r="AX51" s="9" t="n"/>
       <c r="AY51" s="9" t="n"/>
       <c r="AZ51" s="9" t="n"/>
+      <c r="BA51" s="9" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="10" t="n"/>
@@ -4066,6 +4126,7 @@
       <c r="AX52" s="10" t="n"/>
       <c r="AY52" s="10" t="n"/>
       <c r="AZ52" s="10" t="n"/>
+      <c r="BA52" s="10" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="9" t="n"/>
@@ -4120,6 +4181,7 @@
       <c r="AX53" s="9" t="n"/>
       <c r="AY53" s="9" t="n"/>
       <c r="AZ53" s="9" t="n"/>
+      <c r="BA53" s="9" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="n"/>
@@ -4174,6 +4236,7 @@
       <c r="AX54" s="10" t="n"/>
       <c r="AY54" s="10" t="n"/>
       <c r="AZ54" s="10" t="n"/>
+      <c r="BA54" s="10" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="9" t="n"/>
@@ -4228,6 +4291,7 @@
       <c r="AX55" s="9" t="n"/>
       <c r="AY55" s="9" t="n"/>
       <c r="AZ55" s="9" t="n"/>
+      <c r="BA55" s="9" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="10" t="n"/>
@@ -4282,6 +4346,7 @@
       <c r="AX56" s="10" t="n"/>
       <c r="AY56" s="10" t="n"/>
       <c r="AZ56" s="10" t="n"/>
+      <c r="BA56" s="10" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="9" t="n"/>
@@ -4336,6 +4401,7 @@
       <c r="AX57" s="9" t="n"/>
       <c r="AY57" s="9" t="n"/>
       <c r="AZ57" s="9" t="n"/>
+      <c r="BA57" s="9" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="10" t="n"/>
@@ -4390,6 +4456,7 @@
       <c r="AX58" s="10" t="n"/>
       <c r="AY58" s="10" t="n"/>
       <c r="AZ58" s="10" t="n"/>
+      <c r="BA58" s="10" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="9" t="n"/>
@@ -4444,6 +4511,7 @@
       <c r="AX59" s="9" t="n"/>
       <c r="AY59" s="9" t="n"/>
       <c r="AZ59" s="9" t="n"/>
+      <c r="BA59" s="9" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="10" t="n"/>
@@ -4498,6 +4566,7 @@
       <c r="AX60" s="10" t="n"/>
       <c r="AY60" s="10" t="n"/>
       <c r="AZ60" s="10" t="n"/>
+      <c r="BA60" s="10" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="9" t="n"/>
@@ -4552,6 +4621,7 @@
       <c r="AX61" s="9" t="n"/>
       <c r="AY61" s="9" t="n"/>
       <c r="AZ61" s="9" t="n"/>
+      <c r="BA61" s="9" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="10" t="n"/>
@@ -4606,6 +4676,7 @@
       <c r="AX62" s="10" t="n"/>
       <c r="AY62" s="10" t="n"/>
       <c r="AZ62" s="10" t="n"/>
+      <c r="BA62" s="10" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="9" t="n"/>
@@ -4660,6 +4731,7 @@
       <c r="AX63" s="9" t="n"/>
       <c r="AY63" s="9" t="n"/>
       <c r="AZ63" s="9" t="n"/>
+      <c r="BA63" s="9" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="10" t="n"/>
@@ -4714,6 +4786,7 @@
       <c r="AX64" s="10" t="n"/>
       <c r="AY64" s="10" t="n"/>
       <c r="AZ64" s="10" t="n"/>
+      <c r="BA64" s="10" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="9" t="n"/>
@@ -4768,6 +4841,7 @@
       <c r="AX65" s="9" t="n"/>
       <c r="AY65" s="9" t="n"/>
       <c r="AZ65" s="9" t="n"/>
+      <c r="BA65" s="9" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="10" t="n"/>
@@ -4822,6 +4896,7 @@
       <c r="AX66" s="10" t="n"/>
       <c r="AY66" s="10" t="n"/>
       <c r="AZ66" s="10" t="n"/>
+      <c r="BA66" s="10" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="9" t="n"/>
@@ -4876,6 +4951,7 @@
       <c r="AX67" s="9" t="n"/>
       <c r="AY67" s="9" t="n"/>
       <c r="AZ67" s="9" t="n"/>
+      <c r="BA67" s="9" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="10" t="n"/>
@@ -4930,6 +5006,7 @@
       <c r="AX68" s="10" t="n"/>
       <c r="AY68" s="10" t="n"/>
       <c r="AZ68" s="10" t="n"/>
+      <c r="BA68" s="10" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="9" t="n"/>
@@ -4984,6 +5061,7 @@
       <c r="AX69" s="9" t="n"/>
       <c r="AY69" s="9" t="n"/>
       <c r="AZ69" s="9" t="n"/>
+      <c r="BA69" s="9" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="10" t="n"/>
@@ -5038,6 +5116,7 @@
       <c r="AX70" s="10" t="n"/>
       <c r="AY70" s="10" t="n"/>
       <c r="AZ70" s="10" t="n"/>
+      <c r="BA70" s="10" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="9" t="n"/>
@@ -5092,6 +5171,7 @@
       <c r="AX71" s="9" t="n"/>
       <c r="AY71" s="9" t="n"/>
       <c r="AZ71" s="9" t="n"/>
+      <c r="BA71" s="9" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="10" t="n"/>
@@ -5146,6 +5226,7 @@
       <c r="AX72" s="10" t="n"/>
       <c r="AY72" s="10" t="n"/>
       <c r="AZ72" s="10" t="n"/>
+      <c r="BA72" s="10" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="9" t="n"/>
@@ -5200,6 +5281,7 @@
       <c r="AX73" s="9" t="n"/>
       <c r="AY73" s="9" t="n"/>
       <c r="AZ73" s="9" t="n"/>
+      <c r="BA73" s="9" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="10" t="n"/>
@@ -5254,6 +5336,7 @@
       <c r="AX74" s="10" t="n"/>
       <c r="AY74" s="10" t="n"/>
       <c r="AZ74" s="10" t="n"/>
+      <c r="BA74" s="10" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="9" t="n"/>
@@ -5308,6 +5391,7 @@
       <c r="AX75" s="9" t="n"/>
       <c r="AY75" s="9" t="n"/>
       <c r="AZ75" s="9" t="n"/>
+      <c r="BA75" s="9" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="10" t="n"/>
@@ -5362,6 +5446,7 @@
       <c r="AX76" s="10" t="n"/>
       <c r="AY76" s="10" t="n"/>
       <c r="AZ76" s="10" t="n"/>
+      <c r="BA76" s="10" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="9" t="n"/>
@@ -5416,6 +5501,7 @@
       <c r="AX77" s="9" t="n"/>
       <c r="AY77" s="9" t="n"/>
       <c r="AZ77" s="9" t="n"/>
+      <c r="BA77" s="9" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="10" t="n"/>
@@ -5470,6 +5556,7 @@
       <c r="AX78" s="10" t="n"/>
       <c r="AY78" s="10" t="n"/>
       <c r="AZ78" s="10" t="n"/>
+      <c r="BA78" s="10" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="9" t="n"/>
@@ -5524,6 +5611,7 @@
       <c r="AX79" s="9" t="n"/>
       <c r="AY79" s="9" t="n"/>
       <c r="AZ79" s="9" t="n"/>
+      <c r="BA79" s="9" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="10" t="n"/>
@@ -5578,6 +5666,7 @@
       <c r="AX80" s="10" t="n"/>
       <c r="AY80" s="10" t="n"/>
       <c r="AZ80" s="10" t="n"/>
+      <c r="BA80" s="10" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="9" t="n"/>
@@ -5632,6 +5721,7 @@
       <c r="AX81" s="9" t="n"/>
       <c r="AY81" s="9" t="n"/>
       <c r="AZ81" s="9" t="n"/>
+      <c r="BA81" s="9" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="10" t="n"/>
@@ -5686,6 +5776,7 @@
       <c r="AX82" s="10" t="n"/>
       <c r="AY82" s="10" t="n"/>
       <c r="AZ82" s="10" t="n"/>
+      <c r="BA82" s="10" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="9" t="n"/>
@@ -5740,6 +5831,7 @@
       <c r="AX83" s="9" t="n"/>
       <c r="AY83" s="9" t="n"/>
       <c r="AZ83" s="9" t="n"/>
+      <c r="BA83" s="9" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="10" t="n"/>
@@ -5794,6 +5886,7 @@
       <c r="AX84" s="10" t="n"/>
       <c r="AY84" s="10" t="n"/>
       <c r="AZ84" s="10" t="n"/>
+      <c r="BA84" s="10" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="9" t="n"/>
@@ -5848,6 +5941,7 @@
       <c r="AX85" s="9" t="n"/>
       <c r="AY85" s="9" t="n"/>
       <c r="AZ85" s="9" t="n"/>
+      <c r="BA85" s="9" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="10" t="n"/>
@@ -5902,6 +5996,7 @@
       <c r="AX86" s="10" t="n"/>
       <c r="AY86" s="10" t="n"/>
       <c r="AZ86" s="10" t="n"/>
+      <c r="BA86" s="10" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="9" t="n"/>
@@ -5956,6 +6051,7 @@
       <c r="AX87" s="9" t="n"/>
       <c r="AY87" s="9" t="n"/>
       <c r="AZ87" s="9" t="n"/>
+      <c r="BA87" s="9" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="10" t="n"/>
@@ -6010,6 +6106,7 @@
       <c r="AX88" s="10" t="n"/>
       <c r="AY88" s="10" t="n"/>
       <c r="AZ88" s="10" t="n"/>
+      <c r="BA88" s="10" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="9" t="n"/>
@@ -6064,6 +6161,7 @@
       <c r="AX89" s="9" t="n"/>
       <c r="AY89" s="9" t="n"/>
       <c r="AZ89" s="9" t="n"/>
+      <c r="BA89" s="9" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="10" t="n"/>
@@ -6118,6 +6216,7 @@
       <c r="AX90" s="10" t="n"/>
       <c r="AY90" s="10" t="n"/>
       <c r="AZ90" s="10" t="n"/>
+      <c r="BA90" s="10" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="9" t="n"/>
@@ -6172,6 +6271,7 @@
       <c r="AX91" s="9" t="n"/>
       <c r="AY91" s="9" t="n"/>
       <c r="AZ91" s="9" t="n"/>
+      <c r="BA91" s="9" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="10" t="n"/>
@@ -6226,6 +6326,7 @@
       <c r="AX92" s="10" t="n"/>
       <c r="AY92" s="10" t="n"/>
       <c r="AZ92" s="10" t="n"/>
+      <c r="BA92" s="10" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="9" t="n"/>
@@ -6280,6 +6381,7 @@
       <c r="AX93" s="9" t="n"/>
       <c r="AY93" s="9" t="n"/>
       <c r="AZ93" s="9" t="n"/>
+      <c r="BA93" s="9" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="10" t="n"/>
@@ -6334,6 +6436,7 @@
       <c r="AX94" s="10" t="n"/>
       <c r="AY94" s="10" t="n"/>
       <c r="AZ94" s="10" t="n"/>
+      <c r="BA94" s="10" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="9" t="n"/>
@@ -6388,6 +6491,7 @@
       <c r="AX95" s="9" t="n"/>
       <c r="AY95" s="9" t="n"/>
       <c r="AZ95" s="9" t="n"/>
+      <c r="BA95" s="9" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="10" t="n"/>
@@ -6442,6 +6546,7 @@
       <c r="AX96" s="10" t="n"/>
       <c r="AY96" s="10" t="n"/>
       <c r="AZ96" s="10" t="n"/>
+      <c r="BA96" s="10" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="9" t="n"/>
@@ -6496,6 +6601,7 @@
       <c r="AX97" s="9" t="n"/>
       <c r="AY97" s="9" t="n"/>
       <c r="AZ97" s="9" t="n"/>
+      <c r="BA97" s="9" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="10" t="n"/>
@@ -6550,6 +6656,7 @@
       <c r="AX98" s="10" t="n"/>
       <c r="AY98" s="10" t="n"/>
       <c r="AZ98" s="10" t="n"/>
+      <c r="BA98" s="10" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="9" t="n"/>
@@ -6604,6 +6711,7 @@
       <c r="AX99" s="9" t="n"/>
       <c r="AY99" s="9" t="n"/>
       <c r="AZ99" s="9" t="n"/>
+      <c r="BA99" s="9" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="10" t="n"/>
@@ -6658,6 +6766,7 @@
       <c r="AX100" s="10" t="n"/>
       <c r="AY100" s="10" t="n"/>
       <c r="AZ100" s="10" t="n"/>
+      <c r="BA100" s="10" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="9" t="n"/>
@@ -6712,6 +6821,7 @@
       <c r="AX101" s="9" t="n"/>
       <c r="AY101" s="9" t="n"/>
       <c r="AZ101" s="9" t="n"/>
+      <c r="BA101" s="9" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="10" t="n"/>
@@ -6766,18 +6876,19 @@
       <c r="AX102" s="10" t="n"/>
       <c r="AY102" s="10" t="n"/>
       <c r="AZ102" s="10" t="n"/>
+      <c r="BA102" s="10" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AZ2"/>
+  <autoFilter ref="A2:BA2"/>
   <mergeCells count="6">
-    <mergeCell ref="AQ1:AW1"/>
-    <mergeCell ref="AX1:AZ1"/>
     <mergeCell ref="G1:U1"/>
     <mergeCell ref="V1:AD1"/>
     <mergeCell ref="AE1:AP1"/>
+    <mergeCell ref="AY1:BA1"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="AQ1:AX1"/>
   </mergeCells>
-  <dataValidations count="25">
+  <dataValidations count="26">
     <dataValidation sqref="A3:A102" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select a value from the dropdown list." promptTitle="Choose Value" prompt="Select from list" type="list">
       <formula1>"Accessory,Bulbs,Electrical,Grow Lights,High Bays + Low Bays,Indoor Commercial,Indoor Residential,Industrial,Outdoor Commercial,Outdoor Fixtures,Recessed,Tubes"</formula1>
     </dataValidation>
@@ -6847,10 +6958,13 @@
     <dataValidation sqref="AN3:AN102" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select a value from the dropdown list." promptTitle="Choose Value" prompt="Select from list" type="list">
       <formula1>"E12,E26,E39,G5,G13,G24q,GU10,GU24,GU5.3,MR-16,Integrated LED,N/A,Other"</formula1>
     </dataValidation>
-    <dataValidation sqref="AW3:AW102" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select a value from the dropdown list." promptTitle="Choose Value" prompt="Select from list" type="list">
+    <dataValidation sqref="AT3:AT102" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select a value from the dropdown list." promptTitle="Choose Value" prompt="Select from list" type="list">
+      <formula1>"Landed,DDP,DAP,FOB"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AX3:AX102" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select a value from the dropdown list." promptTitle="Choose Value" prompt="Select from list" type="list">
       <formula1>"1-Year,2-Year,3-Year,5-Year,7-Year,10-Year,Lifetime"</formula1>
     </dataValidation>
-    <dataValidation sqref="AY3:AY102" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select a value from the dropdown list." promptTitle="Choose Value" prompt="Select from list" type="list">
+    <dataValidation sqref="AZ3:AZ102" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select a value from the dropdown list." promptTitle="Choose Value" prompt="Select from list" type="list">
       <formula1>"Amazon,Home Depot,Walmart,Lowe's,Direct/Distributor,All"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add Stackline integration + SharePoint local sync path
- Template: "Stackline Data?" Yes/No column at BA, Research Notes shifted to BB
- Instructions: step-by-step Stackline Atlas export, naming convention, upload guide
- Plan: updated architecture, finalized decisions, Step 4 Stackline logic
- SharePoint folder created: PRD Research/Stackline Data/
- Tool reads from local sync: C:\Users\Sunco\Sunco Lighting\Product - Manny Tools\
- Naming convention: Stackline_[Category]_[YYYY-MM]_[type].csv

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/PRD_Research_Template.xlsx
+++ b/templates/PRD_Research_Template.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ideations" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ideations'!$A$2:$BA$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ideations'!$A$2:$BB$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -710,21 +710,21 @@
     <row r="33">
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>RESEARCH GUIDANCE (Columns AY–BA)</t>
+          <t>RESEARCH GUIDANCE (Columns AY–BB)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Known competitors to benchmark, priority sales channels, and any</t>
+          <t xml:space="preserve">  Known competitors to benchmark, priority sales channels, Stackline</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  additional notes or context for the research tool.</t>
+          <t xml:space="preserve">  Data toggle (Yes/No), and additional notes for the research tool.</t>
         </is>
       </c>
     </row>
@@ -763,6 +763,263 @@
       <c r="B41" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  • Row 3 contains an example entry you can overwrite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>STACKLINE DATA (Optional):</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  If you have Stackline Atlas data for the category you’re researching,</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  you can include it to enrich the competitive analysis with Amazon market</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  intelligence (competitor sales, pricing trends, ad spend, traffic data).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  How to use:</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Step 1: Export from Stackline Atlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    a. Log in to Stackline Atlas (atlas.stackline.com)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    b. Navigate to the relevant product segment for your category</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    c. Set the date range to the most recent period (last 12 months recommended)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    d. Click Export → Download CSV</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    e. You will get two files:</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      • Sales data file (contains "_all_" in filename) — revenue, units, market share</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      • Traffic data file (contains "_traffic_" in filename) — ad spend, clicks, conversion</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="3" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Step 2: Rename the files using this convention</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Format:  Stackline_[Category]_[YYYY-MM]_[type].csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="3" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    [Category] = The Category value from Column A (use exact spelling, replace spaces with _)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    [YYYY-MM]  = Year and month of the export (e.g., 2026-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    [type]     = sales  OR  traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="3" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Examples:</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Stackline_Indoor_Commercial_2026-04_sales.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Stackline_Indoor_Commercial_2026-04_traffic.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Stackline_Outdoor_Fixtures_2026-04_sales.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Stackline_Outdoor_Fixtures_2026-04_traffic.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="3" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Step 3: Upload to SharePoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Upload both files to the Product SharePoint site:</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Manny Tools / PRD Research / Stackline Data /</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="3" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Step 4: Mark “Yes” in the Stackline Data? column (Column BA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Set the dropdown to “Yes” for each ideation row where you want</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    the research tool to incorporate Stackline data. The tool will</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    automatically find the newest matching file for the category.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="3" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Note: If multiple exports exist for the same category, the tool picks</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  the most recent one based on the YYYY-MM date in the filename.</t>
         </is>
       </c>
     </row>
@@ -782,7 +1039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA102"/>
+  <dimension ref="A1:BB102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -838,6 +1095,7 @@
     <col width="22" customWidth="1" min="51" max="51"/>
     <col width="22" customWidth="1" min="52" max="52"/>
     <col width="22" customWidth="1" min="53" max="53"/>
+    <col width="22" customWidth="1" min="54" max="54"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -918,6 +1176,7 @@
       </c>
       <c r="AZ1" s="1" t="n"/>
       <c r="BA1" s="1" t="n"/>
+      <c r="BB1" s="1" t="n"/>
     </row>
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
@@ -1181,6 +1440,11 @@
         </is>
       </c>
       <c r="BA2" s="8" t="inlineStr">
+        <is>
+          <t>Stackline Data?</t>
+        </is>
+      </c>
+      <c r="BB2" s="8" t="inlineStr">
         <is>
           <t>Research Notes</t>
         </is>
@@ -1428,6 +1692,11 @@
         </is>
       </c>
       <c r="BA3" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="BB3" s="9" t="inlineStr">
         <is>
           <t>High-output selectable wattage panel to replace PN24-2x4-30W line. Target DLC Premium for utility rebates.</t>
         </is>
@@ -1487,6 +1756,7 @@
       <c r="AY4" s="10" t="n"/>
       <c r="AZ4" s="10" t="n"/>
       <c r="BA4" s="10" t="n"/>
+      <c r="BB4" s="10" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n"/>
@@ -1542,6 +1812,7 @@
       <c r="AY5" s="9" t="n"/>
       <c r="AZ5" s="9" t="n"/>
       <c r="BA5" s="9" t="n"/>
+      <c r="BB5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="10" t="n"/>
@@ -1597,6 +1868,7 @@
       <c r="AY6" s="10" t="n"/>
       <c r="AZ6" s="10" t="n"/>
       <c r="BA6" s="10" t="n"/>
+      <c r="BB6" s="10" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n"/>
@@ -1652,6 +1924,7 @@
       <c r="AY7" s="9" t="n"/>
       <c r="AZ7" s="9" t="n"/>
       <c r="BA7" s="9" t="n"/>
+      <c r="BB7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="n"/>
@@ -1707,6 +1980,7 @@
       <c r="AY8" s="10" t="n"/>
       <c r="AZ8" s="10" t="n"/>
       <c r="BA8" s="10" t="n"/>
+      <c r="BB8" s="10" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="n"/>
@@ -1762,6 +2036,7 @@
       <c r="AY9" s="9" t="n"/>
       <c r="AZ9" s="9" t="n"/>
       <c r="BA9" s="9" t="n"/>
+      <c r="BB9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="n"/>
@@ -1817,6 +2092,7 @@
       <c r="AY10" s="10" t="n"/>
       <c r="AZ10" s="10" t="n"/>
       <c r="BA10" s="10" t="n"/>
+      <c r="BB10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n"/>
@@ -1872,6 +2148,7 @@
       <c r="AY11" s="9" t="n"/>
       <c r="AZ11" s="9" t="n"/>
       <c r="BA11" s="9" t="n"/>
+      <c r="BB11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="n"/>
@@ -1927,6 +2204,7 @@
       <c r="AY12" s="10" t="n"/>
       <c r="AZ12" s="10" t="n"/>
       <c r="BA12" s="10" t="n"/>
+      <c r="BB12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n"/>
@@ -1982,6 +2260,7 @@
       <c r="AY13" s="9" t="n"/>
       <c r="AZ13" s="9" t="n"/>
       <c r="BA13" s="9" t="n"/>
+      <c r="BB13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="n"/>
@@ -2037,6 +2316,7 @@
       <c r="AY14" s="10" t="n"/>
       <c r="AZ14" s="10" t="n"/>
       <c r="BA14" s="10" t="n"/>
+      <c r="BB14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n"/>
@@ -2092,6 +2372,7 @@
       <c r="AY15" s="9" t="n"/>
       <c r="AZ15" s="9" t="n"/>
       <c r="BA15" s="9" t="n"/>
+      <c r="BB15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n"/>
@@ -2147,6 +2428,7 @@
       <c r="AY16" s="10" t="n"/>
       <c r="AZ16" s="10" t="n"/>
       <c r="BA16" s="10" t="n"/>
+      <c r="BB16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="n"/>
@@ -2202,6 +2484,7 @@
       <c r="AY17" s="9" t="n"/>
       <c r="AZ17" s="9" t="n"/>
       <c r="BA17" s="9" t="n"/>
+      <c r="BB17" s="9" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n"/>
@@ -2257,6 +2540,7 @@
       <c r="AY18" s="10" t="n"/>
       <c r="AZ18" s="10" t="n"/>
       <c r="BA18" s="10" t="n"/>
+      <c r="BB18" s="10" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="n"/>
@@ -2312,6 +2596,7 @@
       <c r="AY19" s="9" t="n"/>
       <c r="AZ19" s="9" t="n"/>
       <c r="BA19" s="9" t="n"/>
+      <c r="BB19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n"/>
@@ -2367,6 +2652,7 @@
       <c r="AY20" s="10" t="n"/>
       <c r="AZ20" s="10" t="n"/>
       <c r="BA20" s="10" t="n"/>
+      <c r="BB20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="9" t="n"/>
@@ -2422,6 +2708,7 @@
       <c r="AY21" s="9" t="n"/>
       <c r="AZ21" s="9" t="n"/>
       <c r="BA21" s="9" t="n"/>
+      <c r="BB21" s="9" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n"/>
@@ -2477,6 +2764,7 @@
       <c r="AY22" s="10" t="n"/>
       <c r="AZ22" s="10" t="n"/>
       <c r="BA22" s="10" t="n"/>
+      <c r="BB22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="9" t="n"/>
@@ -2532,6 +2820,7 @@
       <c r="AY23" s="9" t="n"/>
       <c r="AZ23" s="9" t="n"/>
       <c r="BA23" s="9" t="n"/>
+      <c r="BB23" s="9" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n"/>
@@ -2587,6 +2876,7 @@
       <c r="AY24" s="10" t="n"/>
       <c r="AZ24" s="10" t="n"/>
       <c r="BA24" s="10" t="n"/>
+      <c r="BB24" s="10" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="9" t="n"/>
@@ -2642,6 +2932,7 @@
       <c r="AY25" s="9" t="n"/>
       <c r="AZ25" s="9" t="n"/>
       <c r="BA25" s="9" t="n"/>
+      <c r="BB25" s="9" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n"/>
@@ -2697,6 +2988,7 @@
       <c r="AY26" s="10" t="n"/>
       <c r="AZ26" s="10" t="n"/>
       <c r="BA26" s="10" t="n"/>
+      <c r="BB26" s="10" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="9" t="n"/>
@@ -2752,6 +3044,7 @@
       <c r="AY27" s="9" t="n"/>
       <c r="AZ27" s="9" t="n"/>
       <c r="BA27" s="9" t="n"/>
+      <c r="BB27" s="9" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n"/>
@@ -2807,6 +3100,7 @@
       <c r="AY28" s="10" t="n"/>
       <c r="AZ28" s="10" t="n"/>
       <c r="BA28" s="10" t="n"/>
+      <c r="BB28" s="10" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n"/>
@@ -2862,6 +3156,7 @@
       <c r="AY29" s="9" t="n"/>
       <c r="AZ29" s="9" t="n"/>
       <c r="BA29" s="9" t="n"/>
+      <c r="BB29" s="9" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n"/>
@@ -2917,6 +3212,7 @@
       <c r="AY30" s="10" t="n"/>
       <c r="AZ30" s="10" t="n"/>
       <c r="BA30" s="10" t="n"/>
+      <c r="BB30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="9" t="n"/>
@@ -2972,6 +3268,7 @@
       <c r="AY31" s="9" t="n"/>
       <c r="AZ31" s="9" t="n"/>
       <c r="BA31" s="9" t="n"/>
+      <c r="BB31" s="9" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n"/>
@@ -3027,6 +3324,7 @@
       <c r="AY32" s="10" t="n"/>
       <c r="AZ32" s="10" t="n"/>
       <c r="BA32" s="10" t="n"/>
+      <c r="BB32" s="10" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="9" t="n"/>
@@ -3082,6 +3380,7 @@
       <c r="AY33" s="9" t="n"/>
       <c r="AZ33" s="9" t="n"/>
       <c r="BA33" s="9" t="n"/>
+      <c r="BB33" s="9" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="n"/>
@@ -3137,6 +3436,7 @@
       <c r="AY34" s="10" t="n"/>
       <c r="AZ34" s="10" t="n"/>
       <c r="BA34" s="10" t="n"/>
+      <c r="BB34" s="10" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="9" t="n"/>
@@ -3192,6 +3492,7 @@
       <c r="AY35" s="9" t="n"/>
       <c r="AZ35" s="9" t="n"/>
       <c r="BA35" s="9" t="n"/>
+      <c r="BB35" s="9" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="n"/>
@@ -3247,6 +3548,7 @@
       <c r="AY36" s="10" t="n"/>
       <c r="AZ36" s="10" t="n"/>
       <c r="BA36" s="10" t="n"/>
+      <c r="BB36" s="10" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="9" t="n"/>
@@ -3302,6 +3604,7 @@
       <c r="AY37" s="9" t="n"/>
       <c r="AZ37" s="9" t="n"/>
       <c r="BA37" s="9" t="n"/>
+      <c r="BB37" s="9" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="n"/>
@@ -3357,6 +3660,7 @@
       <c r="AY38" s="10" t="n"/>
       <c r="AZ38" s="10" t="n"/>
       <c r="BA38" s="10" t="n"/>
+      <c r="BB38" s="10" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="9" t="n"/>
@@ -3412,6 +3716,7 @@
       <c r="AY39" s="9" t="n"/>
       <c r="AZ39" s="9" t="n"/>
       <c r="BA39" s="9" t="n"/>
+      <c r="BB39" s="9" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="n"/>
@@ -3467,6 +3772,7 @@
       <c r="AY40" s="10" t="n"/>
       <c r="AZ40" s="10" t="n"/>
       <c r="BA40" s="10" t="n"/>
+      <c r="BB40" s="10" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="9" t="n"/>
@@ -3522,6 +3828,7 @@
       <c r="AY41" s="9" t="n"/>
       <c r="AZ41" s="9" t="n"/>
       <c r="BA41" s="9" t="n"/>
+      <c r="BB41" s="9" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="10" t="n"/>
@@ -3577,6 +3884,7 @@
       <c r="AY42" s="10" t="n"/>
       <c r="AZ42" s="10" t="n"/>
       <c r="BA42" s="10" t="n"/>
+      <c r="BB42" s="10" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="9" t="n"/>
@@ -3632,6 +3940,7 @@
       <c r="AY43" s="9" t="n"/>
       <c r="AZ43" s="9" t="n"/>
       <c r="BA43" s="9" t="n"/>
+      <c r="BB43" s="9" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="10" t="n"/>
@@ -3687,6 +3996,7 @@
       <c r="AY44" s="10" t="n"/>
       <c r="AZ44" s="10" t="n"/>
       <c r="BA44" s="10" t="n"/>
+      <c r="BB44" s="10" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="9" t="n"/>
@@ -3742,6 +4052,7 @@
       <c r="AY45" s="9" t="n"/>
       <c r="AZ45" s="9" t="n"/>
       <c r="BA45" s="9" t="n"/>
+      <c r="BB45" s="9" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="10" t="n"/>
@@ -3797,6 +4108,7 @@
       <c r="AY46" s="10" t="n"/>
       <c r="AZ46" s="10" t="n"/>
       <c r="BA46" s="10" t="n"/>
+      <c r="BB46" s="10" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="9" t="n"/>
@@ -3852,6 +4164,7 @@
       <c r="AY47" s="9" t="n"/>
       <c r="AZ47" s="9" t="n"/>
       <c r="BA47" s="9" t="n"/>
+      <c r="BB47" s="9" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="10" t="n"/>
@@ -3907,6 +4220,7 @@
       <c r="AY48" s="10" t="n"/>
       <c r="AZ48" s="10" t="n"/>
       <c r="BA48" s="10" t="n"/>
+      <c r="BB48" s="10" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="9" t="n"/>
@@ -3962,6 +4276,7 @@
       <c r="AY49" s="9" t="n"/>
       <c r="AZ49" s="9" t="n"/>
       <c r="BA49" s="9" t="n"/>
+      <c r="BB49" s="9" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="10" t="n"/>
@@ -4017,6 +4332,7 @@
       <c r="AY50" s="10" t="n"/>
       <c r="AZ50" s="10" t="n"/>
       <c r="BA50" s="10" t="n"/>
+      <c r="BB50" s="10" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="9" t="n"/>
@@ -4072,6 +4388,7 @@
       <c r="AY51" s="9" t="n"/>
       <c r="AZ51" s="9" t="n"/>
       <c r="BA51" s="9" t="n"/>
+      <c r="BB51" s="9" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="10" t="n"/>
@@ -4127,6 +4444,7 @@
       <c r="AY52" s="10" t="n"/>
       <c r="AZ52" s="10" t="n"/>
       <c r="BA52" s="10" t="n"/>
+      <c r="BB52" s="10" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="9" t="n"/>
@@ -4182,6 +4500,7 @@
       <c r="AY53" s="9" t="n"/>
       <c r="AZ53" s="9" t="n"/>
       <c r="BA53" s="9" t="n"/>
+      <c r="BB53" s="9" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="n"/>
@@ -4237,6 +4556,7 @@
       <c r="AY54" s="10" t="n"/>
       <c r="AZ54" s="10" t="n"/>
       <c r="BA54" s="10" t="n"/>
+      <c r="BB54" s="10" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="9" t="n"/>
@@ -4292,6 +4612,7 @@
       <c r="AY55" s="9" t="n"/>
       <c r="AZ55" s="9" t="n"/>
       <c r="BA55" s="9" t="n"/>
+      <c r="BB55" s="9" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="10" t="n"/>
@@ -4347,6 +4668,7 @@
       <c r="AY56" s="10" t="n"/>
       <c r="AZ56" s="10" t="n"/>
       <c r="BA56" s="10" t="n"/>
+      <c r="BB56" s="10" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="9" t="n"/>
@@ -4402,6 +4724,7 @@
       <c r="AY57" s="9" t="n"/>
       <c r="AZ57" s="9" t="n"/>
       <c r="BA57" s="9" t="n"/>
+      <c r="BB57" s="9" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="10" t="n"/>
@@ -4457,6 +4780,7 @@
       <c r="AY58" s="10" t="n"/>
       <c r="AZ58" s="10" t="n"/>
       <c r="BA58" s="10" t="n"/>
+      <c r="BB58" s="10" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="9" t="n"/>
@@ -4512,6 +4836,7 @@
       <c r="AY59" s="9" t="n"/>
       <c r="AZ59" s="9" t="n"/>
       <c r="BA59" s="9" t="n"/>
+      <c r="BB59" s="9" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="10" t="n"/>
@@ -4567,6 +4892,7 @@
       <c r="AY60" s="10" t="n"/>
       <c r="AZ60" s="10" t="n"/>
       <c r="BA60" s="10" t="n"/>
+      <c r="BB60" s="10" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="9" t="n"/>
@@ -4622,6 +4948,7 @@
       <c r="AY61" s="9" t="n"/>
       <c r="AZ61" s="9" t="n"/>
       <c r="BA61" s="9" t="n"/>
+      <c r="BB61" s="9" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="10" t="n"/>
@@ -4677,6 +5004,7 @@
       <c r="AY62" s="10" t="n"/>
       <c r="AZ62" s="10" t="n"/>
       <c r="BA62" s="10" t="n"/>
+      <c r="BB62" s="10" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="9" t="n"/>
@@ -4732,6 +5060,7 @@
       <c r="AY63" s="9" t="n"/>
       <c r="AZ63" s="9" t="n"/>
       <c r="BA63" s="9" t="n"/>
+      <c r="BB63" s="9" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="10" t="n"/>
@@ -4787,6 +5116,7 @@
       <c r="AY64" s="10" t="n"/>
       <c r="AZ64" s="10" t="n"/>
       <c r="BA64" s="10" t="n"/>
+      <c r="BB64" s="10" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="9" t="n"/>
@@ -4842,6 +5172,7 @@
       <c r="AY65" s="9" t="n"/>
       <c r="AZ65" s="9" t="n"/>
       <c r="BA65" s="9" t="n"/>
+      <c r="BB65" s="9" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="10" t="n"/>
@@ -4897,6 +5228,7 @@
       <c r="AY66" s="10" t="n"/>
       <c r="AZ66" s="10" t="n"/>
       <c r="BA66" s="10" t="n"/>
+      <c r="BB66" s="10" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="9" t="n"/>
@@ -4952,6 +5284,7 @@
       <c r="AY67" s="9" t="n"/>
       <c r="AZ67" s="9" t="n"/>
       <c r="BA67" s="9" t="n"/>
+      <c r="BB67" s="9" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="10" t="n"/>
@@ -5007,6 +5340,7 @@
       <c r="AY68" s="10" t="n"/>
       <c r="AZ68" s="10" t="n"/>
       <c r="BA68" s="10" t="n"/>
+      <c r="BB68" s="10" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="9" t="n"/>
@@ -5062,6 +5396,7 @@
       <c r="AY69" s="9" t="n"/>
       <c r="AZ69" s="9" t="n"/>
       <c r="BA69" s="9" t="n"/>
+      <c r="BB69" s="9" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="10" t="n"/>
@@ -5117,6 +5452,7 @@
       <c r="AY70" s="10" t="n"/>
       <c r="AZ70" s="10" t="n"/>
       <c r="BA70" s="10" t="n"/>
+      <c r="BB70" s="10" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="9" t="n"/>
@@ -5172,6 +5508,7 @@
       <c r="AY71" s="9" t="n"/>
       <c r="AZ71" s="9" t="n"/>
       <c r="BA71" s="9" t="n"/>
+      <c r="BB71" s="9" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="10" t="n"/>
@@ -5227,6 +5564,7 @@
       <c r="AY72" s="10" t="n"/>
       <c r="AZ72" s="10" t="n"/>
       <c r="BA72" s="10" t="n"/>
+      <c r="BB72" s="10" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="9" t="n"/>
@@ -5282,6 +5620,7 @@
       <c r="AY73" s="9" t="n"/>
       <c r="AZ73" s="9" t="n"/>
       <c r="BA73" s="9" t="n"/>
+      <c r="BB73" s="9" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="10" t="n"/>
@@ -5337,6 +5676,7 @@
       <c r="AY74" s="10" t="n"/>
       <c r="AZ74" s="10" t="n"/>
       <c r="BA74" s="10" t="n"/>
+      <c r="BB74" s="10" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="9" t="n"/>
@@ -5392,6 +5732,7 @@
       <c r="AY75" s="9" t="n"/>
       <c r="AZ75" s="9" t="n"/>
       <c r="BA75" s="9" t="n"/>
+      <c r="BB75" s="9" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="10" t="n"/>
@@ -5447,6 +5788,7 @@
       <c r="AY76" s="10" t="n"/>
       <c r="AZ76" s="10" t="n"/>
       <c r="BA76" s="10" t="n"/>
+      <c r="BB76" s="10" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="9" t="n"/>
@@ -5502,6 +5844,7 @@
       <c r="AY77" s="9" t="n"/>
       <c r="AZ77" s="9" t="n"/>
       <c r="BA77" s="9" t="n"/>
+      <c r="BB77" s="9" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="10" t="n"/>
@@ -5557,6 +5900,7 @@
       <c r="AY78" s="10" t="n"/>
       <c r="AZ78" s="10" t="n"/>
       <c r="BA78" s="10" t="n"/>
+      <c r="BB78" s="10" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="9" t="n"/>
@@ -5612,6 +5956,7 @@
       <c r="AY79" s="9" t="n"/>
       <c r="AZ79" s="9" t="n"/>
       <c r="BA79" s="9" t="n"/>
+      <c r="BB79" s="9" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="10" t="n"/>
@@ -5667,6 +6012,7 @@
       <c r="AY80" s="10" t="n"/>
       <c r="AZ80" s="10" t="n"/>
       <c r="BA80" s="10" t="n"/>
+      <c r="BB80" s="10" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="9" t="n"/>
@@ -5722,6 +6068,7 @@
       <c r="AY81" s="9" t="n"/>
       <c r="AZ81" s="9" t="n"/>
       <c r="BA81" s="9" t="n"/>
+      <c r="BB81" s="9" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="10" t="n"/>
@@ -5777,6 +6124,7 @@
       <c r="AY82" s="10" t="n"/>
       <c r="AZ82" s="10" t="n"/>
       <c r="BA82" s="10" t="n"/>
+      <c r="BB82" s="10" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="9" t="n"/>
@@ -5832,6 +6180,7 @@
       <c r="AY83" s="9" t="n"/>
       <c r="AZ83" s="9" t="n"/>
       <c r="BA83" s="9" t="n"/>
+      <c r="BB83" s="9" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="10" t="n"/>
@@ -5887,6 +6236,7 @@
       <c r="AY84" s="10" t="n"/>
       <c r="AZ84" s="10" t="n"/>
       <c r="BA84" s="10" t="n"/>
+      <c r="BB84" s="10" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="9" t="n"/>
@@ -5942,6 +6292,7 @@
       <c r="AY85" s="9" t="n"/>
       <c r="AZ85" s="9" t="n"/>
       <c r="BA85" s="9" t="n"/>
+      <c r="BB85" s="9" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="10" t="n"/>
@@ -5997,6 +6348,7 @@
       <c r="AY86" s="10" t="n"/>
       <c r="AZ86" s="10" t="n"/>
       <c r="BA86" s="10" t="n"/>
+      <c r="BB86" s="10" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="9" t="n"/>
@@ -6052,6 +6404,7 @@
       <c r="AY87" s="9" t="n"/>
       <c r="AZ87" s="9" t="n"/>
       <c r="BA87" s="9" t="n"/>
+      <c r="BB87" s="9" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="10" t="n"/>
@@ -6107,6 +6460,7 @@
       <c r="AY88" s="10" t="n"/>
       <c r="AZ88" s="10" t="n"/>
       <c r="BA88" s="10" t="n"/>
+      <c r="BB88" s="10" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="9" t="n"/>
@@ -6162,6 +6516,7 @@
       <c r="AY89" s="9" t="n"/>
       <c r="AZ89" s="9" t="n"/>
       <c r="BA89" s="9" t="n"/>
+      <c r="BB89" s="9" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="10" t="n"/>
@@ -6217,6 +6572,7 @@
       <c r="AY90" s="10" t="n"/>
       <c r="AZ90" s="10" t="n"/>
       <c r="BA90" s="10" t="n"/>
+      <c r="BB90" s="10" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="9" t="n"/>
@@ -6272,6 +6628,7 @@
       <c r="AY91" s="9" t="n"/>
       <c r="AZ91" s="9" t="n"/>
       <c r="BA91" s="9" t="n"/>
+      <c r="BB91" s="9" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="10" t="n"/>
@@ -6327,6 +6684,7 @@
       <c r="AY92" s="10" t="n"/>
       <c r="AZ92" s="10" t="n"/>
       <c r="BA92" s="10" t="n"/>
+      <c r="BB92" s="10" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="9" t="n"/>
@@ -6382,6 +6740,7 @@
       <c r="AY93" s="9" t="n"/>
       <c r="AZ93" s="9" t="n"/>
       <c r="BA93" s="9" t="n"/>
+      <c r="BB93" s="9" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="10" t="n"/>
@@ -6437,6 +6796,7 @@
       <c r="AY94" s="10" t="n"/>
       <c r="AZ94" s="10" t="n"/>
       <c r="BA94" s="10" t="n"/>
+      <c r="BB94" s="10" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="9" t="n"/>
@@ -6492,6 +6852,7 @@
       <c r="AY95" s="9" t="n"/>
       <c r="AZ95" s="9" t="n"/>
       <c r="BA95" s="9" t="n"/>
+      <c r="BB95" s="9" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="10" t="n"/>
@@ -6547,6 +6908,7 @@
       <c r="AY96" s="10" t="n"/>
       <c r="AZ96" s="10" t="n"/>
       <c r="BA96" s="10" t="n"/>
+      <c r="BB96" s="10" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="9" t="n"/>
@@ -6602,6 +6964,7 @@
       <c r="AY97" s="9" t="n"/>
       <c r="AZ97" s="9" t="n"/>
       <c r="BA97" s="9" t="n"/>
+      <c r="BB97" s="9" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="10" t="n"/>
@@ -6657,6 +7020,7 @@
       <c r="AY98" s="10" t="n"/>
       <c r="AZ98" s="10" t="n"/>
       <c r="BA98" s="10" t="n"/>
+      <c r="BB98" s="10" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="9" t="n"/>
@@ -6712,6 +7076,7 @@
       <c r="AY99" s="9" t="n"/>
       <c r="AZ99" s="9" t="n"/>
       <c r="BA99" s="9" t="n"/>
+      <c r="BB99" s="9" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="10" t="n"/>
@@ -6767,6 +7132,7 @@
       <c r="AY100" s="10" t="n"/>
       <c r="AZ100" s="10" t="n"/>
       <c r="BA100" s="10" t="n"/>
+      <c r="BB100" s="10" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="9" t="n"/>
@@ -6822,6 +7188,7 @@
       <c r="AY101" s="9" t="n"/>
       <c r="AZ101" s="9" t="n"/>
       <c r="BA101" s="9" t="n"/>
+      <c r="BB101" s="9" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="10" t="n"/>
@@ -6877,18 +7244,19 @@
       <c r="AY102" s="10" t="n"/>
       <c r="AZ102" s="10" t="n"/>
       <c r="BA102" s="10" t="n"/>
+      <c r="BB102" s="10" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:BA2"/>
+  <autoFilter ref="A2:BB2"/>
   <mergeCells count="6">
+    <mergeCell ref="AY1:BB1"/>
     <mergeCell ref="G1:U1"/>
     <mergeCell ref="V1:AD1"/>
     <mergeCell ref="AE1:AP1"/>
-    <mergeCell ref="AY1:BA1"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="AQ1:AX1"/>
   </mergeCells>
-  <dataValidations count="26">
+  <dataValidations count="27">
     <dataValidation sqref="A3:A102" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select a value from the dropdown list." promptTitle="Choose Value" prompt="Select from list" type="list">
       <formula1>"Accessory,Bulbs,Electrical,Grow Lights,High Bays + Low Bays,Indoor Commercial,Indoor Residential,Industrial,Outdoor Commercial,Outdoor Fixtures,Recessed,Tubes"</formula1>
     </dataValidation>
@@ -6967,6 +7335,9 @@
     <dataValidation sqref="AZ3:AZ102" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select a value from the dropdown list." promptTitle="Choose Value" prompt="Select from list" type="list">
       <formula1>"Amazon,Home Depot,Walmart,Lowe's,Direct/Distributor,All"</formula1>
     </dataValidation>
+    <dataValidation sqref="BA3:BA102" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select a value from the dropdown list." promptTitle="Choose Value" prompt="Select from list" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>